<commit_message>
betterments included after Xindi comments
</commit_message>
<xml_diff>
--- a/02_activities/assignments/top_10_boards_reading_data.xlsx
+++ b/02_activities/assignments/top_10_boards_reading_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabic\DSI\visualization\02_activities\assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6437701-C367-4B14-B885-3CA2E6047CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5C23D4-A1B6-4E97-8D94-E4FC4F15F1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Board Name</t>
   </si>
@@ -57,12 +57,18 @@
   <si>
     <t>Hamilton-Wentworth CDSB</t>
   </si>
+  <si>
+    <t>The table/data above was generated from the Python file assignment-3_Python_code.ipynb</t>
+  </si>
+  <si>
+    <t>To reproduce the chart, select the entire table, click on tab Insert, chart, and select Clustered Bar</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,6 +80,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -111,11 +125,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -148,6 +167,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>G3 Reading Achievement</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -161,11 +205,11 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -179,7 +223,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.18929827905590013"/>
+          <c:y val="8.0861978235515997E-2"/>
+          <c:w val="0.79138452665483849"/>
+          <c:h val="0.83770143180706214"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
@@ -200,14 +254,75 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent1">
+                <a:alpha val="85000"/>
+              </a:schemeClr>
             </a:solidFill>
-            <a:ln>
-              <a:noFill/>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:alpha val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="inEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="50000"/>
+                          <a:lumOff val="50000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$11</c:f>
@@ -292,14 +407,15 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="inEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="182"/>
+        <c:gapWidth val="65"/>
         <c:axId val="879251007"/>
         <c:axId val="879251487"/>
       </c:barChart>
@@ -310,17 +426,72 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-CA"/>
+                  <a:t>Board Name</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+              <a:schemeClr val="dk1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -332,11 +503,11 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -364,17 +535,84 @@
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="95000"/>
+                      <a:lumOff val="5000"/>
+                      <a:alpha val="42000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="0">
+                    <a:schemeClr val="lt1">
+                      <a:lumMod val="75000"/>
+                      <a:alpha val="36000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-CA"/>
+                  <a:t>Average G3 Reading Achievement (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -393,9 +631,9 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -430,14 +668,30 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="39000">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="lt1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="25000"/>
+          <a:lumOff val="75000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:round/>
@@ -503,171 +757,207 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="218">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200" cap="all" baseline="0"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="39000">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
         <a:solidFill>
           <a:schemeClr val="dk1">
             <a:lumMod val="25000"/>
             <a:lumOff val="75000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+          <a:alpha val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
       <a:spAutoFit/>
     </cs:bodyPr>
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
         <a:solidFill>
-          <a:schemeClr val="phClr"/>
+          <a:schemeClr val="phClr">
+            <a:alpha val="85000"/>
+          </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointLine>
   <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -683,21 +973,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -707,18 +995,55 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
@@ -726,108 +1051,183 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
+          <a:schemeClr val="dk1">
             <a:lumMod val="35000"/>
             <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="95000"/>
+          <a:alpha val="39000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
+          <a:schemeClr val="dk1">
             <a:lumMod val="50000"/>
             <a:lumOff val="50000"/>
           </a:schemeClr>
@@ -835,96 +1235,18 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
   </cs:seriesLine>
   <cs:title>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1800" b="1" kern="1200" baseline="0"/>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -933,14 +1255,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -949,9 +1270,9 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -961,20 +1282,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
+          <a:schemeClr val="dk1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -983,11 +1303,16 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -995,14 +1320,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -1011,16 +1330,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>26670</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>125729</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>22859</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>180974</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>60959</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1333,8 +1652,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.21875" customWidth="1"/>
+    <col min="2" max="2" width="35.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -1345,86 +1668,114 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>90.2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>88.384615384615387</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>87.28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <v>85.795454545454547</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>85.296296296296291</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="2">
         <v>83.454545454545453</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="2">
         <v>82.8</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="2">
         <v>80.791666666666671</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="2">
         <v>79.75</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="2">
         <v>79.265306122448976</v>
       </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:B14"/>
+    <mergeCell ref="A16:B17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>